<commit_message>
Solucion de crasheos y arreglo de navegacion para registro
</commit_message>
<xml_diff>
--- a/Doc_Test/Pruebas_Calidad/Pruebas_Unitarias/CEC-10.xlsx
+++ b/Doc_Test/Pruebas_Calidad/Pruebas_Unitarias/CEC-10.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Kevin\Desktop\App_Uv\AppAcompanhamientoUV\Doc_Test\Pruebas_Calidad\Pruebas_Unitarias\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA20E8C3-F03D-4024-A73F-94091B72BD31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73A80B3E-114D-4D2C-A438-EF59D3C64460}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{2FFDA8E8-6428-4D51-9D6D-F314F8731DBF}"/>
   </bookViews>
@@ -945,7 +945,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -969,10 +969,46 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -981,40 +1017,13 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1372,135 +1381,135 @@
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="10" t="s">
+      <c r="C2" s="20" t="s">
         <v>28</v>
       </c>
-      <c r="D2" s="10"/>
-      <c r="E2" s="10"/>
-      <c r="F2" s="10"/>
-      <c r="G2" s="10"/>
-      <c r="H2" s="10"/>
-      <c r="I2" s="10"/>
-      <c r="J2" s="10"/>
-      <c r="K2" s="10"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
+      <c r="F2" s="20"/>
+      <c r="G2" s="20"/>
+      <c r="H2" s="20"/>
+      <c r="I2" s="20"/>
+      <c r="J2" s="20"/>
+      <c r="K2" s="20"/>
     </row>
     <row r="3" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="10" t="s">
+      <c r="C3" s="20" t="s">
         <v>32</v>
       </c>
-      <c r="D3" s="10"/>
-      <c r="E3" s="10"/>
-      <c r="F3" s="10"/>
-      <c r="G3" s="10"/>
-      <c r="H3" s="10"/>
-      <c r="I3" s="10"/>
-      <c r="J3" s="10"/>
-      <c r="K3" s="10"/>
+      <c r="D3" s="20"/>
+      <c r="E3" s="20"/>
+      <c r="F3" s="20"/>
+      <c r="G3" s="20"/>
+      <c r="H3" s="20"/>
+      <c r="I3" s="20"/>
+      <c r="J3" s="20"/>
+      <c r="K3" s="20"/>
     </row>
     <row r="4" spans="2:11" ht="32.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B4" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="9" t="s">
+      <c r="C4" s="21" t="s">
         <v>33</v>
       </c>
-      <c r="D4" s="9"/>
-      <c r="E4" s="9"/>
-      <c r="F4" s="9"/>
-      <c r="G4" s="9"/>
-      <c r="H4" s="9"/>
-      <c r="I4" s="9"/>
-      <c r="J4" s="9"/>
-      <c r="K4" s="9"/>
+      <c r="D4" s="21"/>
+      <c r="E4" s="21"/>
+      <c r="F4" s="21"/>
+      <c r="G4" s="21"/>
+      <c r="H4" s="21"/>
+      <c r="I4" s="21"/>
+      <c r="J4" s="21"/>
+      <c r="K4" s="21"/>
     </row>
     <row r="5" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B5" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="C5" s="14">
+      <c r="C5" s="22">
         <v>45849</v>
       </c>
-      <c r="D5" s="14"/>
-      <c r="E5" s="14"/>
-      <c r="F5" s="14"/>
-      <c r="G5" s="14"/>
-      <c r="H5" s="14"/>
-      <c r="I5" s="14"/>
-      <c r="J5" s="14"/>
-      <c r="K5" s="14"/>
+      <c r="D5" s="22"/>
+      <c r="E5" s="22"/>
+      <c r="F5" s="22"/>
+      <c r="G5" s="22"/>
+      <c r="H5" s="22"/>
+      <c r="I5" s="22"/>
+      <c r="J5" s="22"/>
+      <c r="K5" s="22"/>
     </row>
     <row r="6" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B6" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C6" s="10" t="s">
+      <c r="C6" s="20" t="s">
         <v>29</v>
       </c>
-      <c r="D6" s="10"/>
-      <c r="E6" s="10"/>
-      <c r="F6" s="10"/>
-      <c r="G6" s="10"/>
-      <c r="H6" s="10"/>
-      <c r="I6" s="10"/>
-      <c r="J6" s="10"/>
-      <c r="K6" s="10"/>
+      <c r="D6" s="20"/>
+      <c r="E6" s="20"/>
+      <c r="F6" s="20"/>
+      <c r="G6" s="20"/>
+      <c r="H6" s="20"/>
+      <c r="I6" s="20"/>
+      <c r="J6" s="20"/>
+      <c r="K6" s="20"/>
     </row>
     <row r="7" spans="2:11" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="C7" s="9" t="s">
+      <c r="C7" s="21" t="s">
         <v>30</v>
       </c>
-      <c r="D7" s="9"/>
-      <c r="E7" s="9"/>
-      <c r="F7" s="9"/>
-      <c r="G7" s="9"/>
-      <c r="H7" s="9"/>
-      <c r="I7" s="9"/>
-      <c r="J7" s="9"/>
-      <c r="K7" s="9"/>
+      <c r="D7" s="21"/>
+      <c r="E7" s="21"/>
+      <c r="F7" s="21"/>
+      <c r="G7" s="21"/>
+      <c r="H7" s="21"/>
+      <c r="I7" s="21"/>
+      <c r="J7" s="21"/>
+      <c r="K7" s="21"/>
     </row>
     <row r="8" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B8" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C8" s="10" t="s">
+      <c r="C8" s="20" t="s">
         <v>31</v>
       </c>
-      <c r="D8" s="10"/>
-      <c r="E8" s="10"/>
-      <c r="F8" s="10"/>
-      <c r="G8" s="10"/>
-      <c r="H8" s="10"/>
-      <c r="I8" s="10"/>
-      <c r="J8" s="10"/>
-      <c r="K8" s="10"/>
+      <c r="D8" s="20"/>
+      <c r="E8" s="20"/>
+      <c r="F8" s="20"/>
+      <c r="G8" s="20"/>
+      <c r="H8" s="20"/>
+      <c r="I8" s="20"/>
+      <c r="J8" s="20"/>
+      <c r="K8" s="20"/>
     </row>
     <row r="9" spans="2:11" ht="85.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B9" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C9" s="9" t="s">
+      <c r="C9" s="21" t="s">
         <v>246</v>
       </c>
-      <c r="D9" s="9"/>
-      <c r="E9" s="9"/>
-      <c r="F9" s="9"/>
-      <c r="G9" s="9"/>
-      <c r="H9" s="9"/>
-      <c r="I9" s="9"/>
-      <c r="J9" s="9"/>
-      <c r="K9" s="9"/>
+      <c r="D9" s="21"/>
+      <c r="E9" s="21"/>
+      <c r="F9" s="21"/>
+      <c r="G9" s="21"/>
+      <c r="H9" s="21"/>
+      <c r="I9" s="21"/>
+      <c r="J9" s="21"/>
+      <c r="K9" s="21"/>
     </row>
     <row r="10" spans="2:11" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B10" s="11" t="s">
+      <c r="B10" s="23" t="s">
         <v>5</v>
       </c>
-      <c r="C10" s="12"/>
+      <c r="C10" s="24"/>
       <c r="D10" s="6" t="s">
         <v>6</v>
       </c>
@@ -1527,10 +1536,10 @@
       </c>
     </row>
     <row r="11" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B11" s="15" t="s">
+      <c r="B11" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="C11" s="21" t="s">
+      <c r="C11" s="12" t="s">
         <v>34</v>
       </c>
       <c r="D11" s="13"/>
@@ -1543,8 +1552,8 @@
       <c r="K11" s="13"/>
     </row>
     <row r="12" spans="2:11" ht="54.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="15"/>
-      <c r="C12" s="22" t="s">
+      <c r="B12" s="11"/>
+      <c r="C12" s="10" t="s">
         <v>15</v>
       </c>
       <c r="D12" s="7" t="s">
@@ -1562,17 +1571,17 @@
       <c r="H12" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="I12" s="17" t="s">
+      <c r="I12" s="14" t="s">
         <v>233</v>
       </c>
-      <c r="J12" s="19" t="s">
+      <c r="J12" s="15" t="s">
         <v>62</v>
       </c>
       <c r="K12" s="16"/>
     </row>
     <row r="13" spans="2:11" ht="115.2" x14ac:dyDescent="0.3">
-      <c r="B13" s="15"/>
-      <c r="C13" s="22" t="s">
+      <c r="B13" s="11"/>
+      <c r="C13" s="10" t="s">
         <v>16</v>
       </c>
       <c r="D13" s="3" t="s">
@@ -1590,13 +1599,13 @@
       <c r="H13" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="I13" s="17"/>
-      <c r="J13" s="19"/>
+      <c r="I13" s="14"/>
+      <c r="J13" s="15"/>
       <c r="K13" s="16"/>
     </row>
     <row r="14" spans="2:11" ht="72" x14ac:dyDescent="0.3">
-      <c r="B14" s="15"/>
-      <c r="C14" s="22" t="s">
+      <c r="B14" s="11"/>
+      <c r="C14" s="10" t="s">
         <v>19</v>
       </c>
       <c r="D14" s="3" t="s">
@@ -1614,13 +1623,13 @@
       <c r="H14" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I14" s="17"/>
-      <c r="J14" s="19"/>
+      <c r="I14" s="14"/>
+      <c r="J14" s="15"/>
       <c r="K14" s="16"/>
     </row>
     <row r="15" spans="2:11" ht="72" x14ac:dyDescent="0.3">
-      <c r="B15" s="15"/>
-      <c r="C15" s="22" t="s">
+      <c r="B15" s="11"/>
+      <c r="C15" s="10" t="s">
         <v>63</v>
       </c>
       <c r="D15" s="3" t="s">
@@ -1638,13 +1647,13 @@
       <c r="H15" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I15" s="17"/>
-      <c r="J15" s="19"/>
+      <c r="I15" s="14"/>
+      <c r="J15" s="15"/>
       <c r="K15" s="16"/>
     </row>
     <row r="16" spans="2:11" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="B16" s="15"/>
-      <c r="C16" s="22" t="s">
+      <c r="B16" s="11"/>
+      <c r="C16" s="10" t="s">
         <v>64</v>
       </c>
       <c r="D16" s="3" t="s">
@@ -1662,16 +1671,16 @@
       <c r="H16" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I16" s="17"/>
-      <c r="J16" s="19"/>
+      <c r="I16" s="14"/>
+      <c r="J16" s="15"/>
       <c r="K16" s="16"/>
     </row>
     <row r="17" spans="2:11" ht="72" x14ac:dyDescent="0.3">
-      <c r="B17" s="15"/>
-      <c r="C17" s="22" t="s">
+      <c r="B17" s="11"/>
+      <c r="C17" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="D17" s="18" t="s">
+      <c r="D17" s="9" t="s">
         <v>45</v>
       </c>
       <c r="E17" s="4" t="s">
@@ -1686,13 +1695,13 @@
       <c r="H17" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I17" s="17"/>
-      <c r="J17" s="19"/>
+      <c r="I17" s="14"/>
+      <c r="J17" s="15"/>
       <c r="K17" s="16"/>
     </row>
     <row r="18" spans="2:11" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="B18" s="15"/>
-      <c r="C18" s="22" t="s">
+      <c r="B18" s="11"/>
+      <c r="C18" s="10" t="s">
         <v>66</v>
       </c>
       <c r="D18" s="3" t="s">
@@ -1710,13 +1719,13 @@
       <c r="H18" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I18" s="17"/>
-      <c r="J18" s="19"/>
+      <c r="I18" s="14"/>
+      <c r="J18" s="15"/>
       <c r="K18" s="16"/>
     </row>
     <row r="19" spans="2:11" ht="72" x14ac:dyDescent="0.3">
-      <c r="B19" s="15"/>
-      <c r="C19" s="22" t="s">
+      <c r="B19" s="11"/>
+      <c r="C19" s="10" t="s">
         <v>67</v>
       </c>
       <c r="D19" s="3" t="s">
@@ -1734,13 +1743,13 @@
       <c r="H19" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I19" s="17"/>
-      <c r="J19" s="19"/>
+      <c r="I19" s="14"/>
+      <c r="J19" s="15"/>
       <c r="K19" s="16"/>
     </row>
     <row r="20" spans="2:11" ht="72" x14ac:dyDescent="0.3">
-      <c r="B20" s="15"/>
-      <c r="C20" s="22" t="s">
+      <c r="B20" s="11"/>
+      <c r="C20" s="10" t="s">
         <v>68</v>
       </c>
       <c r="D20" s="3" t="s">
@@ -1758,13 +1767,13 @@
       <c r="H20" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I20" s="17"/>
-      <c r="J20" s="19"/>
+      <c r="I20" s="14"/>
+      <c r="J20" s="15"/>
       <c r="K20" s="16"/>
     </row>
     <row r="21" spans="2:11" ht="72" x14ac:dyDescent="0.3">
-      <c r="B21" s="15"/>
-      <c r="C21" s="22" t="s">
+      <c r="B21" s="11"/>
+      <c r="C21" s="10" t="s">
         <v>69</v>
       </c>
       <c r="D21" s="3" t="s">
@@ -1782,13 +1791,13 @@
       <c r="H21" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I21" s="17"/>
-      <c r="J21" s="19"/>
+      <c r="I21" s="14"/>
+      <c r="J21" s="15"/>
       <c r="K21" s="16"/>
     </row>
     <row r="22" spans="2:11" ht="72" x14ac:dyDescent="0.3">
-      <c r="B22" s="15"/>
-      <c r="C22" s="22" t="s">
+      <c r="B22" s="11"/>
+      <c r="C22" s="10" t="s">
         <v>70</v>
       </c>
       <c r="D22" s="3" t="s">
@@ -1806,13 +1815,13 @@
       <c r="H22" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I22" s="17"/>
-      <c r="J22" s="19"/>
+      <c r="I22" s="14"/>
+      <c r="J22" s="15"/>
       <c r="K22" s="16"/>
     </row>
     <row r="23" spans="2:11" ht="72" x14ac:dyDescent="0.3">
-      <c r="B23" s="15"/>
-      <c r="C23" s="22" t="s">
+      <c r="B23" s="11"/>
+      <c r="C23" s="10" t="s">
         <v>71</v>
       </c>
       <c r="D23" s="3" t="s">
@@ -1830,13 +1839,13 @@
       <c r="H23" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I23" s="17"/>
-      <c r="J23" s="19"/>
+      <c r="I23" s="14"/>
+      <c r="J23" s="15"/>
       <c r="K23" s="16"/>
     </row>
     <row r="24" spans="2:11" ht="72" x14ac:dyDescent="0.3">
-      <c r="B24" s="15"/>
-      <c r="C24" s="22" t="s">
+      <c r="B24" s="11"/>
+      <c r="C24" s="10" t="s">
         <v>72</v>
       </c>
       <c r="D24" s="3" t="s">
@@ -1854,13 +1863,13 @@
       <c r="H24" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I24" s="17"/>
-      <c r="J24" s="19"/>
+      <c r="I24" s="14"/>
+      <c r="J24" s="15"/>
       <c r="K24" s="16"/>
     </row>
     <row r="25" spans="2:11" ht="72" x14ac:dyDescent="0.3">
-      <c r="B25" s="15"/>
-      <c r="C25" s="22" t="s">
+      <c r="B25" s="11"/>
+      <c r="C25" s="10" t="s">
         <v>73</v>
       </c>
       <c r="D25" s="3" t="s">
@@ -1878,13 +1887,13 @@
       <c r="H25" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I25" s="17"/>
-      <c r="J25" s="19"/>
+      <c r="I25" s="14"/>
+      <c r="J25" s="15"/>
       <c r="K25" s="16"/>
     </row>
     <row r="26" spans="2:11" ht="72" x14ac:dyDescent="0.3">
-      <c r="B26" s="15"/>
-      <c r="C26" s="22" t="s">
+      <c r="B26" s="11"/>
+      <c r="C26" s="10" t="s">
         <v>74</v>
       </c>
       <c r="D26" s="3" t="s">
@@ -1902,13 +1911,13 @@
       <c r="H26" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I26" s="17"/>
-      <c r="J26" s="19"/>
+      <c r="I26" s="14"/>
+      <c r="J26" s="15"/>
       <c r="K26" s="16"/>
     </row>
     <row r="27" spans="2:11" ht="72" x14ac:dyDescent="0.3">
-      <c r="B27" s="15"/>
-      <c r="C27" s="22" t="s">
+      <c r="B27" s="11"/>
+      <c r="C27" s="10" t="s">
         <v>75</v>
       </c>
       <c r="D27" s="3" t="s">
@@ -1926,13 +1935,13 @@
       <c r="H27" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I27" s="17"/>
-      <c r="J27" s="19"/>
+      <c r="I27" s="14"/>
+      <c r="J27" s="15"/>
       <c r="K27" s="16"/>
     </row>
     <row r="28" spans="2:11" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B28" s="15"/>
-      <c r="C28" s="22" t="s">
+      <c r="B28" s="11"/>
+      <c r="C28" s="10" t="s">
         <v>76</v>
       </c>
       <c r="D28" s="3" t="s">
@@ -1950,13 +1959,13 @@
       <c r="H28" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I28" s="17"/>
-      <c r="J28" s="19"/>
+      <c r="I28" s="14"/>
+      <c r="J28" s="15"/>
       <c r="K28" s="16"/>
     </row>
     <row r="29" spans="2:11" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B29" s="15"/>
-      <c r="C29" s="22" t="s">
+      <c r="B29" s="11"/>
+      <c r="C29" s="10" t="s">
         <v>77</v>
       </c>
       <c r="D29" s="3" t="s">
@@ -1974,15 +1983,15 @@
       <c r="H29" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I29" s="17"/>
-      <c r="J29" s="20"/>
+      <c r="I29" s="14"/>
+      <c r="J29" s="19"/>
       <c r="K29" s="16"/>
     </row>
     <row r="30" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B30" s="15" t="s">
+      <c r="B30" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="C30" s="21" t="s">
+      <c r="C30" s="12" t="s">
         <v>78</v>
       </c>
       <c r="D30" s="13"/>
@@ -1995,8 +2004,8 @@
       <c r="K30" s="13"/>
     </row>
     <row r="31" spans="2:11" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="B31" s="15"/>
-      <c r="C31" s="22" t="s">
+      <c r="B31" s="11"/>
+      <c r="C31" s="10" t="s">
         <v>25</v>
       </c>
       <c r="D31" s="7" t="s">
@@ -2014,17 +2023,17 @@
       <c r="H31" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="I31" s="17" t="s">
+      <c r="I31" s="14" t="s">
         <v>233</v>
       </c>
-      <c r="J31" s="19" t="s">
+      <c r="J31" s="15" t="s">
         <v>62</v>
       </c>
       <c r="K31" s="16"/>
     </row>
     <row r="32" spans="2:11" ht="115.2" x14ac:dyDescent="0.3">
-      <c r="B32" s="15"/>
-      <c r="C32" s="22" t="s">
+      <c r="B32" s="11"/>
+      <c r="C32" s="10" t="s">
         <v>26</v>
       </c>
       <c r="D32" s="3" t="s">
@@ -2042,13 +2051,13 @@
       <c r="H32" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="I32" s="17"/>
-      <c r="J32" s="19"/>
+      <c r="I32" s="14"/>
+      <c r="J32" s="15"/>
       <c r="K32" s="16"/>
     </row>
     <row r="33" spans="2:11" ht="72" x14ac:dyDescent="0.3">
-      <c r="B33" s="15"/>
-      <c r="C33" s="22" t="s">
+      <c r="B33" s="11"/>
+      <c r="C33" s="10" t="s">
         <v>27</v>
       </c>
       <c r="D33" s="3" t="s">
@@ -2066,13 +2075,13 @@
       <c r="H33" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I33" s="17"/>
-      <c r="J33" s="19"/>
+      <c r="I33" s="14"/>
+      <c r="J33" s="15"/>
       <c r="K33" s="16"/>
     </row>
     <row r="34" spans="2:11" ht="72" x14ac:dyDescent="0.3">
-      <c r="B34" s="15"/>
-      <c r="C34" s="22" t="s">
+      <c r="B34" s="11"/>
+      <c r="C34" s="10" t="s">
         <v>92</v>
       </c>
       <c r="D34" s="3" t="s">
@@ -2090,13 +2099,13 @@
       <c r="H34" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I34" s="17"/>
-      <c r="J34" s="19"/>
+      <c r="I34" s="14"/>
+      <c r="J34" s="15"/>
       <c r="K34" s="16"/>
     </row>
     <row r="35" spans="2:11" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="B35" s="15"/>
-      <c r="C35" s="22" t="s">
+      <c r="B35" s="11"/>
+      <c r="C35" s="10" t="s">
         <v>93</v>
       </c>
       <c r="D35" s="3" t="s">
@@ -2114,13 +2123,13 @@
       <c r="H35" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I35" s="17"/>
-      <c r="J35" s="19"/>
+      <c r="I35" s="14"/>
+      <c r="J35" s="15"/>
       <c r="K35" s="16"/>
     </row>
     <row r="36" spans="2:11" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="B36" s="15"/>
-      <c r="C36" s="22" t="s">
+      <c r="B36" s="11"/>
+      <c r="C36" s="10" t="s">
         <v>94</v>
       </c>
       <c r="D36" s="3" t="s">
@@ -2138,13 +2147,13 @@
       <c r="H36" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I36" s="17"/>
-      <c r="J36" s="19"/>
+      <c r="I36" s="14"/>
+      <c r="J36" s="15"/>
       <c r="K36" s="16"/>
     </row>
     <row r="37" spans="2:11" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B37" s="15"/>
-      <c r="C37" s="22" t="s">
+      <c r="B37" s="11"/>
+      <c r="C37" s="10" t="s">
         <v>95</v>
       </c>
       <c r="D37" s="3" t="s">
@@ -2162,13 +2171,13 @@
       <c r="H37" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I37" s="17"/>
-      <c r="J37" s="19"/>
+      <c r="I37" s="14"/>
+      <c r="J37" s="15"/>
       <c r="K37" s="16"/>
     </row>
     <row r="38" spans="2:11" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B38" s="15"/>
-      <c r="C38" s="22" t="s">
+      <c r="B38" s="11"/>
+      <c r="C38" s="10" t="s">
         <v>96</v>
       </c>
       <c r="D38" s="3" t="s">
@@ -2186,13 +2195,13 @@
       <c r="H38" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I38" s="17"/>
-      <c r="J38" s="19"/>
+      <c r="I38" s="14"/>
+      <c r="J38" s="15"/>
       <c r="K38" s="16"/>
     </row>
     <row r="39" spans="2:11" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B39" s="15"/>
-      <c r="C39" s="22" t="s">
+      <c r="B39" s="11"/>
+      <c r="C39" s="10" t="s">
         <v>97</v>
       </c>
       <c r="D39" s="3" t="s">
@@ -2210,13 +2219,13 @@
       <c r="H39" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I39" s="17"/>
-      <c r="J39" s="19"/>
+      <c r="I39" s="14"/>
+      <c r="J39" s="15"/>
       <c r="K39" s="16"/>
     </row>
     <row r="40" spans="2:11" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B40" s="15"/>
-      <c r="C40" s="22" t="s">
+      <c r="B40" s="11"/>
+      <c r="C40" s="10" t="s">
         <v>98</v>
       </c>
       <c r="D40" s="3" t="s">
@@ -2234,13 +2243,13 @@
       <c r="H40" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I40" s="17"/>
-      <c r="J40" s="19"/>
+      <c r="I40" s="14"/>
+      <c r="J40" s="15"/>
       <c r="K40" s="16"/>
     </row>
     <row r="41" spans="2:11" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B41" s="15"/>
-      <c r="C41" s="22" t="s">
+      <c r="B41" s="11"/>
+      <c r="C41" s="10" t="s">
         <v>99</v>
       </c>
       <c r="D41" s="3" t="s">
@@ -2258,13 +2267,13 @@
       <c r="H41" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I41" s="17"/>
-      <c r="J41" s="19"/>
+      <c r="I41" s="14"/>
+      <c r="J41" s="15"/>
       <c r="K41" s="16"/>
     </row>
     <row r="42" spans="2:11" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B42" s="15"/>
-      <c r="C42" s="22" t="s">
+      <c r="B42" s="11"/>
+      <c r="C42" s="10" t="s">
         <v>100</v>
       </c>
       <c r="D42" s="3" t="s">
@@ -2282,13 +2291,13 @@
       <c r="H42" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I42" s="17"/>
-      <c r="J42" s="19"/>
+      <c r="I42" s="14"/>
+      <c r="J42" s="15"/>
       <c r="K42" s="16"/>
     </row>
     <row r="43" spans="2:11" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B43" s="15"/>
-      <c r="C43" s="22" t="s">
+      <c r="B43" s="11"/>
+      <c r="C43" s="10" t="s">
         <v>101</v>
       </c>
       <c r="D43" s="3" t="s">
@@ -2306,13 +2315,13 @@
       <c r="H43" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I43" s="17"/>
-      <c r="J43" s="19"/>
+      <c r="I43" s="14"/>
+      <c r="J43" s="15"/>
       <c r="K43" s="16"/>
     </row>
     <row r="44" spans="2:11" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B44" s="15"/>
-      <c r="C44" s="22" t="s">
+      <c r="B44" s="11"/>
+      <c r="C44" s="10" t="s">
         <v>102</v>
       </c>
       <c r="D44" s="3" t="s">
@@ -2330,13 +2339,13 @@
       <c r="H44" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I44" s="17"/>
-      <c r="J44" s="19"/>
+      <c r="I44" s="14"/>
+      <c r="J44" s="15"/>
       <c r="K44" s="16"/>
     </row>
     <row r="45" spans="2:11" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B45" s="15"/>
-      <c r="C45" s="22" t="s">
+      <c r="B45" s="11"/>
+      <c r="C45" s="10" t="s">
         <v>103</v>
       </c>
       <c r="D45" s="3" t="s">
@@ -2354,13 +2363,13 @@
       <c r="H45" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I45" s="17"/>
-      <c r="J45" s="19"/>
+      <c r="I45" s="14"/>
+      <c r="J45" s="15"/>
       <c r="K45" s="16"/>
     </row>
     <row r="46" spans="2:11" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B46" s="15"/>
-      <c r="C46" s="22" t="s">
+      <c r="B46" s="11"/>
+      <c r="C46" s="10" t="s">
         <v>104</v>
       </c>
       <c r="D46" s="3" t="s">
@@ -2378,13 +2387,13 @@
       <c r="H46" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I46" s="17"/>
-      <c r="J46" s="19"/>
+      <c r="I46" s="14"/>
+      <c r="J46" s="15"/>
       <c r="K46" s="16"/>
     </row>
     <row r="47" spans="2:11" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B47" s="15"/>
-      <c r="C47" s="22" t="s">
+      <c r="B47" s="11"/>
+      <c r="C47" s="10" t="s">
         <v>105</v>
       </c>
       <c r="D47" s="3" t="s">
@@ -2402,15 +2411,15 @@
       <c r="H47" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I47" s="17"/>
-      <c r="J47" s="20"/>
+      <c r="I47" s="14"/>
+      <c r="J47" s="19"/>
       <c r="K47" s="16"/>
     </row>
     <row r="48" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B48" s="15" t="s">
+      <c r="B48" s="11" t="s">
         <v>109</v>
       </c>
-      <c r="C48" s="21" t="s">
+      <c r="C48" s="12" t="s">
         <v>106</v>
       </c>
       <c r="D48" s="13"/>
@@ -2423,8 +2432,8 @@
       <c r="K48" s="13"/>
     </row>
     <row r="49" spans="2:11" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="B49" s="15"/>
-      <c r="C49" s="22" t="s">
+      <c r="B49" s="11"/>
+      <c r="C49" s="10" t="s">
         <v>110</v>
       </c>
       <c r="D49" s="7" t="s">
@@ -2442,17 +2451,17 @@
       <c r="H49" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="I49" s="17" t="s">
+      <c r="I49" s="14" t="s">
         <v>233</v>
       </c>
-      <c r="J49" s="19" t="s">
+      <c r="J49" s="15" t="s">
         <v>62</v>
       </c>
       <c r="K49" s="16"/>
     </row>
     <row r="50" spans="2:11" ht="115.2" x14ac:dyDescent="0.3">
-      <c r="B50" s="15"/>
-      <c r="C50" s="22" t="s">
+      <c r="B50" s="11"/>
+      <c r="C50" s="10" t="s">
         <v>111</v>
       </c>
       <c r="D50" s="3" t="s">
@@ -2470,13 +2479,13 @@
       <c r="H50" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="I50" s="17"/>
-      <c r="J50" s="19"/>
+      <c r="I50" s="14"/>
+      <c r="J50" s="15"/>
       <c r="K50" s="16"/>
     </row>
     <row r="51" spans="2:11" ht="72" x14ac:dyDescent="0.3">
-      <c r="B51" s="15"/>
-      <c r="C51" s="22" t="s">
+      <c r="B51" s="11"/>
+      <c r="C51" s="10" t="s">
         <v>112</v>
       </c>
       <c r="D51" s="3" t="s">
@@ -2494,13 +2503,13 @@
       <c r="H51" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I51" s="17"/>
-      <c r="J51" s="19"/>
+      <c r="I51" s="14"/>
+      <c r="J51" s="15"/>
       <c r="K51" s="16"/>
     </row>
     <row r="52" spans="2:11" ht="72" x14ac:dyDescent="0.3">
-      <c r="B52" s="15"/>
-      <c r="C52" s="22" t="s">
+      <c r="B52" s="11"/>
+      <c r="C52" s="10" t="s">
         <v>113</v>
       </c>
       <c r="D52" s="3" t="s">
@@ -2518,13 +2527,13 @@
       <c r="H52" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I52" s="17"/>
-      <c r="J52" s="19"/>
+      <c r="I52" s="14"/>
+      <c r="J52" s="15"/>
       <c r="K52" s="16"/>
     </row>
     <row r="53" spans="2:11" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="B53" s="15"/>
-      <c r="C53" s="22" t="s">
+      <c r="B53" s="11"/>
+      <c r="C53" s="10" t="s">
         <v>114</v>
       </c>
       <c r="D53" s="3" t="s">
@@ -2542,13 +2551,13 @@
       <c r="H53" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I53" s="17"/>
-      <c r="J53" s="19"/>
+      <c r="I53" s="14"/>
+      <c r="J53" s="15"/>
       <c r="K53" s="16"/>
     </row>
     <row r="54" spans="2:11" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="B54" s="15"/>
-      <c r="C54" s="22" t="s">
+      <c r="B54" s="11"/>
+      <c r="C54" s="10" t="s">
         <v>115</v>
       </c>
       <c r="D54" s="3" t="s">
@@ -2566,13 +2575,13 @@
       <c r="H54" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I54" s="17"/>
-      <c r="J54" s="19"/>
+      <c r="I54" s="14"/>
+      <c r="J54" s="15"/>
       <c r="K54" s="16"/>
     </row>
     <row r="55" spans="2:11" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B55" s="15"/>
-      <c r="C55" s="22" t="s">
+      <c r="B55" s="11"/>
+      <c r="C55" s="10" t="s">
         <v>116</v>
       </c>
       <c r="D55" s="3" t="s">
@@ -2590,13 +2599,13 @@
       <c r="H55" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I55" s="17"/>
-      <c r="J55" s="19"/>
+      <c r="I55" s="14"/>
+      <c r="J55" s="15"/>
       <c r="K55" s="16"/>
     </row>
     <row r="56" spans="2:11" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B56" s="15"/>
-      <c r="C56" s="22" t="s">
+      <c r="B56" s="11"/>
+      <c r="C56" s="10" t="s">
         <v>117</v>
       </c>
       <c r="D56" s="3" t="s">
@@ -2614,13 +2623,13 @@
       <c r="H56" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I56" s="17"/>
-      <c r="J56" s="19"/>
+      <c r="I56" s="14"/>
+      <c r="J56" s="15"/>
       <c r="K56" s="16"/>
     </row>
     <row r="57" spans="2:11" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B57" s="15"/>
-      <c r="C57" s="22" t="s">
+      <c r="B57" s="11"/>
+      <c r="C57" s="10" t="s">
         <v>118</v>
       </c>
       <c r="D57" s="3" t="s">
@@ -2638,13 +2647,13 @@
       <c r="H57" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I57" s="17"/>
-      <c r="J57" s="19"/>
+      <c r="I57" s="14"/>
+      <c r="J57" s="15"/>
       <c r="K57" s="16"/>
     </row>
     <row r="58" spans="2:11" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B58" s="15"/>
-      <c r="C58" s="22" t="s">
+      <c r="B58" s="11"/>
+      <c r="C58" s="10" t="s">
         <v>119</v>
       </c>
       <c r="D58" s="3" t="s">
@@ -2662,13 +2671,13 @@
       <c r="H58" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I58" s="17"/>
-      <c r="J58" s="19"/>
+      <c r="I58" s="14"/>
+      <c r="J58" s="15"/>
       <c r="K58" s="16"/>
     </row>
     <row r="59" spans="2:11" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B59" s="15"/>
-      <c r="C59" s="22" t="s">
+      <c r="B59" s="11"/>
+      <c r="C59" s="10" t="s">
         <v>120</v>
       </c>
       <c r="D59" s="3" t="s">
@@ -2686,13 +2695,13 @@
       <c r="H59" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I59" s="17"/>
-      <c r="J59" s="19"/>
+      <c r="I59" s="14"/>
+      <c r="J59" s="15"/>
       <c r="K59" s="16"/>
     </row>
     <row r="60" spans="2:11" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B60" s="15"/>
-      <c r="C60" s="22" t="s">
+      <c r="B60" s="11"/>
+      <c r="C60" s="10" t="s">
         <v>121</v>
       </c>
       <c r="D60" s="3" t="s">
@@ -2710,13 +2719,13 @@
       <c r="H60" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I60" s="17"/>
-      <c r="J60" s="19"/>
+      <c r="I60" s="14"/>
+      <c r="J60" s="15"/>
       <c r="K60" s="16"/>
     </row>
     <row r="61" spans="2:11" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B61" s="15"/>
-      <c r="C61" s="22" t="s">
+      <c r="B61" s="11"/>
+      <c r="C61" s="10" t="s">
         <v>122</v>
       </c>
       <c r="D61" s="3" t="s">
@@ -2734,13 +2743,13 @@
       <c r="H61" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I61" s="17"/>
-      <c r="J61" s="19"/>
+      <c r="I61" s="14"/>
+      <c r="J61" s="15"/>
       <c r="K61" s="16"/>
     </row>
     <row r="62" spans="2:11" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B62" s="15"/>
-      <c r="C62" s="22" t="s">
+      <c r="B62" s="11"/>
+      <c r="C62" s="10" t="s">
         <v>123</v>
       </c>
       <c r="D62" s="3" t="s">
@@ -2758,13 +2767,13 @@
       <c r="H62" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I62" s="17"/>
-      <c r="J62" s="19"/>
+      <c r="I62" s="14"/>
+      <c r="J62" s="15"/>
       <c r="K62" s="16"/>
     </row>
     <row r="63" spans="2:11" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B63" s="15"/>
-      <c r="C63" s="22" t="s">
+      <c r="B63" s="11"/>
+      <c r="C63" s="10" t="s">
         <v>124</v>
       </c>
       <c r="D63" s="3" t="s">
@@ -2782,13 +2791,13 @@
       <c r="H63" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I63" s="17"/>
-      <c r="J63" s="19"/>
+      <c r="I63" s="14"/>
+      <c r="J63" s="15"/>
       <c r="K63" s="16"/>
     </row>
     <row r="64" spans="2:11" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="B64" s="15"/>
-      <c r="C64" s="22" t="s">
+      <c r="B64" s="11"/>
+      <c r="C64" s="10" t="s">
         <v>125</v>
       </c>
       <c r="D64" s="3" t="s">
@@ -2806,13 +2815,13 @@
       <c r="H64" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I64" s="17"/>
-      <c r="J64" s="19"/>
+      <c r="I64" s="14"/>
+      <c r="J64" s="15"/>
       <c r="K64" s="16"/>
     </row>
     <row r="65" spans="2:11" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B65" s="15"/>
-      <c r="C65" s="22" t="s">
+      <c r="B65" s="11"/>
+      <c r="C65" s="10" t="s">
         <v>126</v>
       </c>
       <c r="D65" s="3" t="s">
@@ -2830,15 +2839,15 @@
       <c r="H65" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I65" s="17"/>
-      <c r="J65" s="20"/>
+      <c r="I65" s="14"/>
+      <c r="J65" s="19"/>
       <c r="K65" s="16"/>
     </row>
     <row r="66" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B66" s="15" t="s">
+      <c r="B66" s="11" t="s">
         <v>132</v>
       </c>
-      <c r="C66" s="21" t="s">
+      <c r="C66" s="12" t="s">
         <v>127</v>
       </c>
       <c r="D66" s="13"/>
@@ -2851,8 +2860,8 @@
       <c r="K66" s="13"/>
     </row>
     <row r="67" spans="2:11" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="B67" s="15"/>
-      <c r="C67" s="22" t="s">
+      <c r="B67" s="11"/>
+      <c r="C67" s="10" t="s">
         <v>133</v>
       </c>
       <c r="D67" s="7" t="s">
@@ -2870,17 +2879,17 @@
       <c r="H67" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="I67" s="17" t="s">
+      <c r="I67" s="14" t="s">
         <v>233</v>
       </c>
-      <c r="J67" s="19" t="s">
+      <c r="J67" s="15" t="s">
         <v>62</v>
       </c>
       <c r="K67" s="16"/>
     </row>
     <row r="68" spans="2:11" ht="115.2" x14ac:dyDescent="0.3">
-      <c r="B68" s="15"/>
-      <c r="C68" s="22" t="s">
+      <c r="B68" s="11"/>
+      <c r="C68" s="10" t="s">
         <v>134</v>
       </c>
       <c r="D68" s="3" t="s">
@@ -2898,13 +2907,13 @@
       <c r="H68" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="I68" s="17"/>
-      <c r="J68" s="19"/>
+      <c r="I68" s="14"/>
+      <c r="J68" s="15"/>
       <c r="K68" s="16"/>
     </row>
     <row r="69" spans="2:11" ht="72" x14ac:dyDescent="0.3">
-      <c r="B69" s="15"/>
-      <c r="C69" s="22" t="s">
+      <c r="B69" s="11"/>
+      <c r="C69" s="10" t="s">
         <v>135</v>
       </c>
       <c r="D69" s="3" t="s">
@@ -2922,13 +2931,13 @@
       <c r="H69" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I69" s="17"/>
-      <c r="J69" s="19"/>
+      <c r="I69" s="14"/>
+      <c r="J69" s="15"/>
       <c r="K69" s="16"/>
     </row>
     <row r="70" spans="2:11" ht="72" x14ac:dyDescent="0.3">
-      <c r="B70" s="15"/>
-      <c r="C70" s="22" t="s">
+      <c r="B70" s="11"/>
+      <c r="C70" s="10" t="s">
         <v>136</v>
       </c>
       <c r="D70" s="3" t="s">
@@ -2946,13 +2955,13 @@
       <c r="H70" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I70" s="17"/>
-      <c r="J70" s="19"/>
+      <c r="I70" s="14"/>
+      <c r="J70" s="15"/>
       <c r="K70" s="16"/>
     </row>
     <row r="71" spans="2:11" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="B71" s="15"/>
-      <c r="C71" s="22" t="s">
+      <c r="B71" s="11"/>
+      <c r="C71" s="10" t="s">
         <v>137</v>
       </c>
       <c r="D71" s="3" t="s">
@@ -2970,13 +2979,13 @@
       <c r="H71" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I71" s="17"/>
-      <c r="J71" s="19"/>
+      <c r="I71" s="14"/>
+      <c r="J71" s="15"/>
       <c r="K71" s="16"/>
     </row>
     <row r="72" spans="2:11" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="B72" s="15"/>
-      <c r="C72" s="22" t="s">
+      <c r="B72" s="11"/>
+      <c r="C72" s="10" t="s">
         <v>138</v>
       </c>
       <c r="D72" s="3" t="s">
@@ -2994,13 +3003,13 @@
       <c r="H72" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I72" s="17"/>
-      <c r="J72" s="19"/>
+      <c r="I72" s="14"/>
+      <c r="J72" s="15"/>
       <c r="K72" s="16"/>
     </row>
     <row r="73" spans="2:11" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B73" s="15"/>
-      <c r="C73" s="22" t="s">
+      <c r="B73" s="11"/>
+      <c r="C73" s="10" t="s">
         <v>139</v>
       </c>
       <c r="D73" s="3" t="s">
@@ -3018,13 +3027,13 @@
       <c r="H73" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I73" s="17"/>
-      <c r="J73" s="19"/>
+      <c r="I73" s="14"/>
+      <c r="J73" s="15"/>
       <c r="K73" s="16"/>
     </row>
     <row r="74" spans="2:11" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B74" s="15"/>
-      <c r="C74" s="22" t="s">
+      <c r="B74" s="11"/>
+      <c r="C74" s="10" t="s">
         <v>140</v>
       </c>
       <c r="D74" s="3" t="s">
@@ -3042,13 +3051,13 @@
       <c r="H74" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I74" s="17"/>
-      <c r="J74" s="19"/>
+      <c r="I74" s="14"/>
+      <c r="J74" s="15"/>
       <c r="K74" s="16"/>
     </row>
     <row r="75" spans="2:11" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B75" s="15"/>
-      <c r="C75" s="22" t="s">
+      <c r="B75" s="11"/>
+      <c r="C75" s="10" t="s">
         <v>141</v>
       </c>
       <c r="D75" s="3" t="s">
@@ -3066,13 +3075,13 @@
       <c r="H75" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I75" s="17"/>
-      <c r="J75" s="19"/>
+      <c r="I75" s="14"/>
+      <c r="J75" s="15"/>
       <c r="K75" s="16"/>
     </row>
     <row r="76" spans="2:11" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B76" s="15"/>
-      <c r="C76" s="22" t="s">
+      <c r="B76" s="11"/>
+      <c r="C76" s="10" t="s">
         <v>142</v>
       </c>
       <c r="D76" s="3" t="s">
@@ -3090,13 +3099,13 @@
       <c r="H76" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I76" s="17"/>
-      <c r="J76" s="19"/>
+      <c r="I76" s="14"/>
+      <c r="J76" s="15"/>
       <c r="K76" s="16"/>
     </row>
     <row r="77" spans="2:11" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B77" s="15"/>
-      <c r="C77" s="22" t="s">
+      <c r="B77" s="11"/>
+      <c r="C77" s="10" t="s">
         <v>143</v>
       </c>
       <c r="D77" s="3" t="s">
@@ -3114,13 +3123,13 @@
       <c r="H77" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I77" s="17"/>
-      <c r="J77" s="19"/>
+      <c r="I77" s="14"/>
+      <c r="J77" s="15"/>
       <c r="K77" s="16"/>
     </row>
     <row r="78" spans="2:11" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B78" s="15"/>
-      <c r="C78" s="22" t="s">
+      <c r="B78" s="11"/>
+      <c r="C78" s="10" t="s">
         <v>144</v>
       </c>
       <c r="D78" s="3" t="s">
@@ -3138,13 +3147,13 @@
       <c r="H78" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I78" s="17"/>
-      <c r="J78" s="19"/>
+      <c r="I78" s="14"/>
+      <c r="J78" s="15"/>
       <c r="K78" s="16"/>
     </row>
     <row r="79" spans="2:11" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B79" s="15"/>
-      <c r="C79" s="22" t="s">
+      <c r="B79" s="11"/>
+      <c r="C79" s="10" t="s">
         <v>145</v>
       </c>
       <c r="D79" s="3" t="s">
@@ -3162,13 +3171,13 @@
       <c r="H79" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I79" s="17"/>
-      <c r="J79" s="19"/>
+      <c r="I79" s="14"/>
+      <c r="J79" s="15"/>
       <c r="K79" s="16"/>
     </row>
     <row r="80" spans="2:11" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B80" s="15"/>
-      <c r="C80" s="22" t="s">
+      <c r="B80" s="11"/>
+      <c r="C80" s="10" t="s">
         <v>146</v>
       </c>
       <c r="D80" s="3" t="s">
@@ -3186,13 +3195,13 @@
       <c r="H80" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I80" s="17"/>
-      <c r="J80" s="19"/>
+      <c r="I80" s="14"/>
+      <c r="J80" s="15"/>
       <c r="K80" s="16"/>
     </row>
     <row r="81" spans="2:11" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B81" s="15"/>
-      <c r="C81" s="22" t="s">
+      <c r="B81" s="11"/>
+      <c r="C81" s="10" t="s">
         <v>147</v>
       </c>
       <c r="D81" s="3" t="s">
@@ -3210,13 +3219,13 @@
       <c r="H81" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I81" s="17"/>
-      <c r="J81" s="19"/>
+      <c r="I81" s="14"/>
+      <c r="J81" s="15"/>
       <c r="K81" s="16"/>
     </row>
     <row r="82" spans="2:11" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B82" s="15"/>
-      <c r="C82" s="22" t="s">
+      <c r="B82" s="11"/>
+      <c r="C82" s="10" t="s">
         <v>148</v>
       </c>
       <c r="D82" s="3" t="s">
@@ -3234,13 +3243,13 @@
       <c r="H82" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I82" s="17"/>
-      <c r="J82" s="19"/>
+      <c r="I82" s="14"/>
+      <c r="J82" s="15"/>
       <c r="K82" s="16"/>
     </row>
     <row r="83" spans="2:11" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B83" s="15"/>
-      <c r="C83" s="22" t="s">
+      <c r="B83" s="11"/>
+      <c r="C83" s="10" t="s">
         <v>149</v>
       </c>
       <c r="D83" s="3" t="s">
@@ -3258,15 +3267,15 @@
       <c r="H83" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I83" s="17"/>
-      <c r="J83" s="20"/>
+      <c r="I83" s="14"/>
+      <c r="J83" s="19"/>
       <c r="K83" s="16"/>
     </row>
     <row r="84" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B84" s="15" t="s">
+      <c r="B84" s="11" t="s">
         <v>152</v>
       </c>
-      <c r="C84" s="21" t="s">
+      <c r="C84" s="12" t="s">
         <v>150</v>
       </c>
       <c r="D84" s="13"/>
@@ -3279,8 +3288,8 @@
       <c r="K84" s="13"/>
     </row>
     <row r="85" spans="2:11" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="B85" s="15"/>
-      <c r="C85" s="22" t="s">
+      <c r="B85" s="11"/>
+      <c r="C85" s="10" t="s">
         <v>153</v>
       </c>
       <c r="D85" s="7" t="s">
@@ -3298,17 +3307,17 @@
       <c r="H85" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="I85" s="17" t="s">
+      <c r="I85" s="14" t="s">
         <v>233</v>
       </c>
-      <c r="J85" s="19" t="s">
+      <c r="J85" s="15" t="s">
         <v>62</v>
       </c>
       <c r="K85" s="16"/>
     </row>
     <row r="86" spans="2:11" ht="115.2" x14ac:dyDescent="0.3">
-      <c r="B86" s="15"/>
-      <c r="C86" s="22" t="s">
+      <c r="B86" s="11"/>
+      <c r="C86" s="10" t="s">
         <v>154</v>
       </c>
       <c r="D86" s="3" t="s">
@@ -3326,13 +3335,13 @@
       <c r="H86" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="I86" s="17"/>
-      <c r="J86" s="19"/>
+      <c r="I86" s="14"/>
+      <c r="J86" s="15"/>
       <c r="K86" s="16"/>
     </row>
     <row r="87" spans="2:11" ht="72" x14ac:dyDescent="0.3">
-      <c r="B87" s="15"/>
-      <c r="C87" s="22" t="s">
+      <c r="B87" s="11"/>
+      <c r="C87" s="10" t="s">
         <v>155</v>
       </c>
       <c r="D87" s="3" t="s">
@@ -3350,13 +3359,13 @@
       <c r="H87" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I87" s="17"/>
-      <c r="J87" s="19"/>
+      <c r="I87" s="14"/>
+      <c r="J87" s="15"/>
       <c r="K87" s="16"/>
     </row>
     <row r="88" spans="2:11" ht="72" x14ac:dyDescent="0.3">
-      <c r="B88" s="15"/>
-      <c r="C88" s="22" t="s">
+      <c r="B88" s="11"/>
+      <c r="C88" s="10" t="s">
         <v>156</v>
       </c>
       <c r="D88" s="3" t="s">
@@ -3374,13 +3383,13 @@
       <c r="H88" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I88" s="17"/>
-      <c r="J88" s="19"/>
+      <c r="I88" s="14"/>
+      <c r="J88" s="15"/>
       <c r="K88" s="16"/>
     </row>
     <row r="89" spans="2:11" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="B89" s="15"/>
-      <c r="C89" s="22" t="s">
+      <c r="B89" s="11"/>
+      <c r="C89" s="10" t="s">
         <v>157</v>
       </c>
       <c r="D89" s="3" t="s">
@@ -3398,13 +3407,13 @@
       <c r="H89" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I89" s="17"/>
-      <c r="J89" s="19"/>
+      <c r="I89" s="14"/>
+      <c r="J89" s="15"/>
       <c r="K89" s="16"/>
     </row>
     <row r="90" spans="2:11" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="B90" s="15"/>
-      <c r="C90" s="22" t="s">
+      <c r="B90" s="11"/>
+      <c r="C90" s="10" t="s">
         <v>158</v>
       </c>
       <c r="D90" s="3" t="s">
@@ -3422,13 +3431,13 @@
       <c r="H90" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I90" s="17"/>
-      <c r="J90" s="19"/>
+      <c r="I90" s="14"/>
+      <c r="J90" s="15"/>
       <c r="K90" s="16"/>
     </row>
     <row r="91" spans="2:11" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B91" s="15"/>
-      <c r="C91" s="22" t="s">
+      <c r="B91" s="11"/>
+      <c r="C91" s="10" t="s">
         <v>159</v>
       </c>
       <c r="D91" s="3" t="s">
@@ -3446,13 +3455,13 @@
       <c r="H91" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I91" s="17"/>
-      <c r="J91" s="19"/>
+      <c r="I91" s="14"/>
+      <c r="J91" s="15"/>
       <c r="K91" s="16"/>
     </row>
     <row r="92" spans="2:11" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B92" s="15"/>
-      <c r="C92" s="22" t="s">
+      <c r="B92" s="11"/>
+      <c r="C92" s="10" t="s">
         <v>160</v>
       </c>
       <c r="D92" s="3" t="s">
@@ -3470,13 +3479,13 @@
       <c r="H92" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I92" s="17"/>
-      <c r="J92" s="19"/>
+      <c r="I92" s="14"/>
+      <c r="J92" s="15"/>
       <c r="K92" s="16"/>
     </row>
     <row r="93" spans="2:11" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B93" s="15"/>
-      <c r="C93" s="22" t="s">
+      <c r="B93" s="11"/>
+      <c r="C93" s="10" t="s">
         <v>161</v>
       </c>
       <c r="D93" s="3" t="s">
@@ -3494,13 +3503,13 @@
       <c r="H93" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I93" s="17"/>
-      <c r="J93" s="19"/>
+      <c r="I93" s="14"/>
+      <c r="J93" s="15"/>
       <c r="K93" s="16"/>
     </row>
     <row r="94" spans="2:11" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B94" s="15"/>
-      <c r="C94" s="22" t="s">
+      <c r="B94" s="11"/>
+      <c r="C94" s="10" t="s">
         <v>162</v>
       </c>
       <c r="D94" s="3" t="s">
@@ -3518,13 +3527,13 @@
       <c r="H94" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I94" s="17"/>
-      <c r="J94" s="19"/>
+      <c r="I94" s="14"/>
+      <c r="J94" s="15"/>
       <c r="K94" s="16"/>
     </row>
     <row r="95" spans="2:11" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B95" s="15"/>
-      <c r="C95" s="22" t="s">
+      <c r="B95" s="11"/>
+      <c r="C95" s="10" t="s">
         <v>163</v>
       </c>
       <c r="D95" s="3" t="s">
@@ -3542,13 +3551,13 @@
       <c r="H95" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I95" s="17"/>
-      <c r="J95" s="19"/>
+      <c r="I95" s="14"/>
+      <c r="J95" s="15"/>
       <c r="K95" s="16"/>
     </row>
     <row r="96" spans="2:11" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B96" s="15"/>
-      <c r="C96" s="22" t="s">
+      <c r="B96" s="11"/>
+      <c r="C96" s="10" t="s">
         <v>164</v>
       </c>
       <c r="D96" s="3" t="s">
@@ -3566,13 +3575,13 @@
       <c r="H96" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I96" s="17"/>
-      <c r="J96" s="19"/>
+      <c r="I96" s="14"/>
+      <c r="J96" s="15"/>
       <c r="K96" s="16"/>
     </row>
     <row r="97" spans="2:11" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B97" s="15"/>
-      <c r="C97" s="22" t="s">
+      <c r="B97" s="11"/>
+      <c r="C97" s="10" t="s">
         <v>165</v>
       </c>
       <c r="D97" s="3" t="s">
@@ -3590,13 +3599,13 @@
       <c r="H97" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I97" s="17"/>
-      <c r="J97" s="19"/>
+      <c r="I97" s="14"/>
+      <c r="J97" s="15"/>
       <c r="K97" s="16"/>
     </row>
     <row r="98" spans="2:11" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B98" s="15"/>
-      <c r="C98" s="22" t="s">
+      <c r="B98" s="11"/>
+      <c r="C98" s="10" t="s">
         <v>166</v>
       </c>
       <c r="D98" s="3" t="s">
@@ -3614,13 +3623,13 @@
       <c r="H98" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I98" s="17"/>
-      <c r="J98" s="19"/>
+      <c r="I98" s="14"/>
+      <c r="J98" s="15"/>
       <c r="K98" s="16"/>
     </row>
     <row r="99" spans="2:11" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B99" s="15"/>
-      <c r="C99" s="22" t="s">
+      <c r="B99" s="11"/>
+      <c r="C99" s="10" t="s">
         <v>167</v>
       </c>
       <c r="D99" s="3" t="s">
@@ -3638,13 +3647,13 @@
       <c r="H99" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I99" s="17"/>
-      <c r="J99" s="19"/>
+      <c r="I99" s="14"/>
+      <c r="J99" s="15"/>
       <c r="K99" s="16"/>
     </row>
     <row r="100" spans="2:11" ht="72" x14ac:dyDescent="0.3">
-      <c r="B100" s="15"/>
-      <c r="C100" s="22" t="s">
+      <c r="B100" s="11"/>
+      <c r="C100" s="10" t="s">
         <v>168</v>
       </c>
       <c r="D100" s="3" t="s">
@@ -3662,13 +3671,13 @@
       <c r="H100" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I100" s="17"/>
-      <c r="J100" s="19"/>
+      <c r="I100" s="14"/>
+      <c r="J100" s="15"/>
       <c r="K100" s="16"/>
     </row>
     <row r="101" spans="2:11" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B101" s="15"/>
-      <c r="C101" s="22" t="s">
+      <c r="B101" s="11"/>
+      <c r="C101" s="10" t="s">
         <v>169</v>
       </c>
       <c r="D101" s="3" t="s">
@@ -3686,15 +3695,15 @@
       <c r="H101" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I101" s="17"/>
-      <c r="J101" s="20"/>
+      <c r="I101" s="14"/>
+      <c r="J101" s="19"/>
       <c r="K101" s="16"/>
     </row>
     <row r="102" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B102" s="15" t="s">
+      <c r="B102" s="11" t="s">
         <v>187</v>
       </c>
-      <c r="C102" s="21" t="s">
+      <c r="C102" s="12" t="s">
         <v>170</v>
       </c>
       <c r="D102" s="13"/>
@@ -3707,8 +3716,8 @@
       <c r="K102" s="13"/>
     </row>
     <row r="103" spans="2:11" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="B103" s="15"/>
-      <c r="C103" s="22" t="s">
+      <c r="B103" s="11"/>
+      <c r="C103" s="10" t="s">
         <v>188</v>
       </c>
       <c r="D103" s="7" t="s">
@@ -3726,19 +3735,19 @@
       <c r="H103" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="I103" s="23" t="s">
+      <c r="I103" s="17" t="s">
         <v>234</v>
       </c>
-      <c r="J103" s="19" t="s">
+      <c r="J103" s="15" t="s">
         <v>62</v>
       </c>
-      <c r="K103" s="23" t="s">
+      <c r="K103" s="17" t="s">
         <v>186</v>
       </c>
     </row>
     <row r="104" spans="2:11" ht="115.2" x14ac:dyDescent="0.3">
-      <c r="B104" s="15"/>
-      <c r="C104" s="22" t="s">
+      <c r="B104" s="11"/>
+      <c r="C104" s="10" t="s">
         <v>189</v>
       </c>
       <c r="D104" s="3" t="s">
@@ -3756,13 +3765,13 @@
       <c r="H104" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="I104" s="23"/>
-      <c r="J104" s="19"/>
-      <c r="K104" s="23"/>
+      <c r="I104" s="17"/>
+      <c r="J104" s="15"/>
+      <c r="K104" s="17"/>
     </row>
     <row r="105" spans="2:11" ht="72" x14ac:dyDescent="0.3">
-      <c r="B105" s="15"/>
-      <c r="C105" s="22" t="s">
+      <c r="B105" s="11"/>
+      <c r="C105" s="10" t="s">
         <v>190</v>
       </c>
       <c r="D105" s="3" t="s">
@@ -3780,13 +3789,13 @@
       <c r="H105" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I105" s="23"/>
-      <c r="J105" s="19"/>
-      <c r="K105" s="23"/>
+      <c r="I105" s="17"/>
+      <c r="J105" s="15"/>
+      <c r="K105" s="17"/>
     </row>
     <row r="106" spans="2:11" ht="72" x14ac:dyDescent="0.3">
-      <c r="B106" s="15"/>
-      <c r="C106" s="22" t="s">
+      <c r="B106" s="11"/>
+      <c r="C106" s="10" t="s">
         <v>191</v>
       </c>
       <c r="D106" s="3" t="s">
@@ -3804,13 +3813,13 @@
       <c r="H106" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I106" s="23"/>
-      <c r="J106" s="19"/>
-      <c r="K106" s="23"/>
+      <c r="I106" s="17"/>
+      <c r="J106" s="15"/>
+      <c r="K106" s="17"/>
     </row>
     <row r="107" spans="2:11" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B107" s="15"/>
-      <c r="C107" s="22" t="s">
+      <c r="B107" s="11"/>
+      <c r="C107" s="10" t="s">
         <v>192</v>
       </c>
       <c r="D107" s="3" t="s">
@@ -3828,13 +3837,13 @@
       <c r="H107" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I107" s="23"/>
-      <c r="J107" s="19"/>
-      <c r="K107" s="23"/>
+      <c r="I107" s="17"/>
+      <c r="J107" s="15"/>
+      <c r="K107" s="17"/>
     </row>
     <row r="108" spans="2:11" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="B108" s="15"/>
-      <c r="C108" s="22" t="s">
+      <c r="B108" s="11"/>
+      <c r="C108" s="10" t="s">
         <v>193</v>
       </c>
       <c r="D108" s="3" t="s">
@@ -3852,13 +3861,13 @@
       <c r="H108" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I108" s="23"/>
-      <c r="J108" s="19"/>
-      <c r="K108" s="23"/>
+      <c r="I108" s="17"/>
+      <c r="J108" s="15"/>
+      <c r="K108" s="17"/>
     </row>
     <row r="109" spans="2:11" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B109" s="15"/>
-      <c r="C109" s="22" t="s">
+      <c r="B109" s="11"/>
+      <c r="C109" s="10" t="s">
         <v>194</v>
       </c>
       <c r="D109" s="3" t="s">
@@ -3876,13 +3885,13 @@
       <c r="H109" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I109" s="23"/>
-      <c r="J109" s="19"/>
-      <c r="K109" s="23"/>
+      <c r="I109" s="17"/>
+      <c r="J109" s="15"/>
+      <c r="K109" s="17"/>
     </row>
     <row r="110" spans="2:11" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B110" s="15"/>
-      <c r="C110" s="22" t="s">
+      <c r="B110" s="11"/>
+      <c r="C110" s="10" t="s">
         <v>195</v>
       </c>
       <c r="D110" s="3" t="s">
@@ -3900,13 +3909,13 @@
       <c r="H110" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I110" s="23"/>
-      <c r="J110" s="19"/>
-      <c r="K110" s="23"/>
+      <c r="I110" s="17"/>
+      <c r="J110" s="15"/>
+      <c r="K110" s="17"/>
     </row>
     <row r="111" spans="2:11" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B111" s="15"/>
-      <c r="C111" s="22" t="s">
+      <c r="B111" s="11"/>
+      <c r="C111" s="10" t="s">
         <v>196</v>
       </c>
       <c r="D111" s="3" t="s">
@@ -3924,13 +3933,13 @@
       <c r="H111" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I111" s="23"/>
-      <c r="J111" s="19"/>
-      <c r="K111" s="23"/>
+      <c r="I111" s="17"/>
+      <c r="J111" s="15"/>
+      <c r="K111" s="17"/>
     </row>
     <row r="112" spans="2:11" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B112" s="15"/>
-      <c r="C112" s="22" t="s">
+      <c r="B112" s="11"/>
+      <c r="C112" s="10" t="s">
         <v>197</v>
       </c>
       <c r="D112" s="3" t="s">
@@ -3948,13 +3957,13 @@
       <c r="H112" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I112" s="23"/>
-      <c r="J112" s="19"/>
-      <c r="K112" s="23"/>
+      <c r="I112" s="17"/>
+      <c r="J112" s="15"/>
+      <c r="K112" s="17"/>
     </row>
     <row r="113" spans="2:11" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B113" s="15"/>
-      <c r="C113" s="22" t="s">
+      <c r="B113" s="11"/>
+      <c r="C113" s="10" t="s">
         <v>198</v>
       </c>
       <c r="D113" s="3" t="s">
@@ -3972,13 +3981,13 @@
       <c r="H113" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I113" s="23"/>
-      <c r="J113" s="19"/>
-      <c r="K113" s="23"/>
+      <c r="I113" s="17"/>
+      <c r="J113" s="15"/>
+      <c r="K113" s="17"/>
     </row>
     <row r="114" spans="2:11" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B114" s="15"/>
-      <c r="C114" s="22" t="s">
+      <c r="B114" s="11"/>
+      <c r="C114" s="10" t="s">
         <v>199</v>
       </c>
       <c r="D114" s="3" t="s">
@@ -3996,13 +4005,13 @@
       <c r="H114" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I114" s="23"/>
-      <c r="J114" s="19"/>
-      <c r="K114" s="23"/>
+      <c r="I114" s="17"/>
+      <c r="J114" s="15"/>
+      <c r="K114" s="17"/>
     </row>
     <row r="115" spans="2:11" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B115" s="15"/>
-      <c r="C115" s="22" t="s">
+      <c r="B115" s="11"/>
+      <c r="C115" s="10" t="s">
         <v>200</v>
       </c>
       <c r="D115" s="3" t="s">
@@ -4020,13 +4029,13 @@
       <c r="H115" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I115" s="23"/>
-      <c r="J115" s="19"/>
-      <c r="K115" s="23"/>
+      <c r="I115" s="17"/>
+      <c r="J115" s="15"/>
+      <c r="K115" s="17"/>
     </row>
     <row r="116" spans="2:11" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B116" s="15"/>
-      <c r="C116" s="22" t="s">
+      <c r="B116" s="11"/>
+      <c r="C116" s="10" t="s">
         <v>201</v>
       </c>
       <c r="D116" s="3" t="s">
@@ -4044,13 +4053,13 @@
       <c r="H116" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I116" s="23"/>
-      <c r="J116" s="19"/>
-      <c r="K116" s="23"/>
+      <c r="I116" s="17"/>
+      <c r="J116" s="15"/>
+      <c r="K116" s="17"/>
     </row>
     <row r="117" spans="2:11" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B117" s="15"/>
-      <c r="C117" s="22" t="s">
+      <c r="B117" s="11"/>
+      <c r="C117" s="10" t="s">
         <v>202</v>
       </c>
       <c r="D117" s="3" t="s">
@@ -4068,13 +4077,13 @@
       <c r="H117" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I117" s="23"/>
-      <c r="J117" s="19"/>
-      <c r="K117" s="23"/>
+      <c r="I117" s="17"/>
+      <c r="J117" s="15"/>
+      <c r="K117" s="17"/>
     </row>
     <row r="118" spans="2:11" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="B118" s="15"/>
-      <c r="C118" s="22" t="s">
+      <c r="B118" s="11"/>
+      <c r="C118" s="10" t="s">
         <v>203</v>
       </c>
       <c r="D118" s="3" t="s">
@@ -4092,13 +4101,13 @@
       <c r="H118" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I118" s="23"/>
-      <c r="J118" s="19"/>
-      <c r="K118" s="23"/>
+      <c r="I118" s="17"/>
+      <c r="J118" s="15"/>
+      <c r="K118" s="17"/>
     </row>
     <row r="119" spans="2:11" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B119" s="15"/>
-      <c r="C119" s="22" t="s">
+      <c r="B119" s="11"/>
+      <c r="C119" s="10" t="s">
         <v>204</v>
       </c>
       <c r="D119" s="3" t="s">
@@ -4116,13 +4125,13 @@
       <c r="H119" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I119" s="23"/>
-      <c r="J119" s="19"/>
-      <c r="K119" s="23"/>
+      <c r="I119" s="17"/>
+      <c r="J119" s="15"/>
+      <c r="K119" s="17"/>
     </row>
     <row r="120" spans="2:11" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B120" s="15"/>
-      <c r="C120" s="22" t="s">
+      <c r="B120" s="11"/>
+      <c r="C120" s="10" t="s">
         <v>205</v>
       </c>
       <c r="D120" s="3" t="s">
@@ -4140,13 +4149,13 @@
       <c r="H120" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I120" s="23"/>
-      <c r="J120" s="19"/>
-      <c r="K120" s="23"/>
+      <c r="I120" s="17"/>
+      <c r="J120" s="15"/>
+      <c r="K120" s="17"/>
     </row>
     <row r="121" spans="2:11" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="B121" s="15"/>
-      <c r="C121" s="22" t="s">
+      <c r="B121" s="11"/>
+      <c r="C121" s="10" t="s">
         <v>206</v>
       </c>
       <c r="D121" s="3" t="s">
@@ -4164,13 +4173,13 @@
       <c r="H121" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I121" s="23"/>
-      <c r="J121" s="19"/>
-      <c r="K121" s="23"/>
+      <c r="I121" s="17"/>
+      <c r="J121" s="15"/>
+      <c r="K121" s="17"/>
     </row>
     <row r="122" spans="2:11" ht="86.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B122" s="15"/>
-      <c r="C122" s="22" t="s">
+      <c r="B122" s="11"/>
+      <c r="C122" s="10" t="s">
         <v>207</v>
       </c>
       <c r="D122" s="3" t="s">
@@ -4188,13 +4197,13 @@
       <c r="H122" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I122" s="23"/>
-      <c r="J122" s="19"/>
-      <c r="K122" s="23"/>
+      <c r="I122" s="17"/>
+      <c r="J122" s="15"/>
+      <c r="K122" s="17"/>
     </row>
     <row r="123" spans="2:11" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="B123" s="15"/>
-      <c r="C123" s="22" t="s">
+      <c r="B123" s="11"/>
+      <c r="C123" s="10" t="s">
         <v>208</v>
       </c>
       <c r="D123" s="3" t="s">
@@ -4212,13 +4221,13 @@
       <c r="H123" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I123" s="23"/>
-      <c r="J123" s="19"/>
-      <c r="K123" s="23"/>
+      <c r="I123" s="17"/>
+      <c r="J123" s="15"/>
+      <c r="K123" s="17"/>
     </row>
     <row r="124" spans="2:11" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="B124" s="15"/>
-      <c r="C124" s="22" t="s">
+      <c r="B124" s="11"/>
+      <c r="C124" s="10" t="s">
         <v>209</v>
       </c>
       <c r="D124" s="3" t="s">
@@ -4236,13 +4245,13 @@
       <c r="H124" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I124" s="23"/>
-      <c r="J124" s="19"/>
-      <c r="K124" s="23"/>
+      <c r="I124" s="17"/>
+      <c r="J124" s="15"/>
+      <c r="K124" s="17"/>
     </row>
     <row r="125" spans="2:11" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="B125" s="15"/>
-      <c r="C125" s="22" t="s">
+      <c r="B125" s="11"/>
+      <c r="C125" s="10" t="s">
         <v>210</v>
       </c>
       <c r="D125" s="3" t="s">
@@ -4260,13 +4269,13 @@
       <c r="H125" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I125" s="23"/>
-      <c r="J125" s="19"/>
-      <c r="K125" s="23"/>
+      <c r="I125" s="17"/>
+      <c r="J125" s="15"/>
+      <c r="K125" s="17"/>
     </row>
     <row r="126" spans="2:11" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B126" s="15"/>
-      <c r="C126" s="22" t="s">
+      <c r="B126" s="11"/>
+      <c r="C126" s="10" t="s">
         <v>211</v>
       </c>
       <c r="D126" s="3" t="s">
@@ -4284,15 +4293,15 @@
       <c r="H126" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I126" s="24"/>
-      <c r="J126" s="20"/>
-      <c r="K126" s="24"/>
+      <c r="I126" s="18"/>
+      <c r="J126" s="19"/>
+      <c r="K126" s="18"/>
     </row>
     <row r="127" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B127" s="15" t="s">
+      <c r="B127" s="11" t="s">
         <v>218</v>
       </c>
-      <c r="C127" s="21" t="s">
+      <c r="C127" s="12" t="s">
         <v>212</v>
       </c>
       <c r="D127" s="13"/>
@@ -4305,8 +4314,8 @@
       <c r="K127" s="13"/>
     </row>
     <row r="128" spans="2:11" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="B128" s="15"/>
-      <c r="C128" s="22" t="s">
+      <c r="B128" s="11"/>
+      <c r="C128" s="10" t="s">
         <v>219</v>
       </c>
       <c r="D128" s="7" t="s">
@@ -4324,17 +4333,17 @@
       <c r="H128" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="I128" s="17" t="s">
+      <c r="I128" s="14" t="s">
         <v>233</v>
       </c>
-      <c r="J128" s="19" t="s">
+      <c r="J128" s="15" t="s">
         <v>62</v>
       </c>
       <c r="K128" s="16"/>
     </row>
     <row r="129" spans="2:11" ht="115.2" x14ac:dyDescent="0.3">
-      <c r="B129" s="15"/>
-      <c r="C129" s="22" t="s">
+      <c r="B129" s="11"/>
+      <c r="C129" s="10" t="s">
         <v>220</v>
       </c>
       <c r="D129" s="3" t="s">
@@ -4352,13 +4361,13 @@
       <c r="H129" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="I129" s="17"/>
-      <c r="J129" s="19"/>
+      <c r="I129" s="14"/>
+      <c r="J129" s="15"/>
       <c r="K129" s="16"/>
     </row>
     <row r="130" spans="2:11" ht="72" x14ac:dyDescent="0.3">
-      <c r="B130" s="15"/>
-      <c r="C130" s="22" t="s">
+      <c r="B130" s="11"/>
+      <c r="C130" s="10" t="s">
         <v>221</v>
       </c>
       <c r="D130" s="3" t="s">
@@ -4376,13 +4385,13 @@
       <c r="H130" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I130" s="17"/>
-      <c r="J130" s="19"/>
+      <c r="I130" s="14"/>
+      <c r="J130" s="15"/>
       <c r="K130" s="16"/>
     </row>
     <row r="131" spans="2:11" ht="72" x14ac:dyDescent="0.3">
-      <c r="B131" s="15"/>
-      <c r="C131" s="22" t="s">
+      <c r="B131" s="11"/>
+      <c r="C131" s="10" t="s">
         <v>222</v>
       </c>
       <c r="D131" s="3" t="s">
@@ -4400,13 +4409,13 @@
       <c r="H131" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I131" s="17"/>
-      <c r="J131" s="19"/>
+      <c r="I131" s="14"/>
+      <c r="J131" s="15"/>
       <c r="K131" s="16"/>
     </row>
     <row r="132" spans="2:11" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="B132" s="15"/>
-      <c r="C132" s="22" t="s">
+      <c r="B132" s="11"/>
+      <c r="C132" s="10" t="s">
         <v>223</v>
       </c>
       <c r="D132" s="3" t="s">
@@ -4424,16 +4433,16 @@
       <c r="H132" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I132" s="17"/>
-      <c r="J132" s="19"/>
+      <c r="I132" s="14"/>
+      <c r="J132" s="15"/>
       <c r="K132" s="16"/>
     </row>
     <row r="133" spans="2:11" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B133" s="15"/>
-      <c r="C133" s="22" t="s">
+      <c r="B133" s="11"/>
+      <c r="C133" s="10" t="s">
         <v>224</v>
       </c>
-      <c r="D133" s="18" t="s">
+      <c r="D133" s="9" t="s">
         <v>213</v>
       </c>
       <c r="E133" s="4" t="s">
@@ -4448,13 +4457,13 @@
       <c r="H133" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I133" s="17"/>
-      <c r="J133" s="19"/>
+      <c r="I133" s="14"/>
+      <c r="J133" s="15"/>
       <c r="K133" s="16"/>
     </row>
     <row r="134" spans="2:11" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B134" s="15"/>
-      <c r="C134" s="22" t="s">
+      <c r="B134" s="11"/>
+      <c r="C134" s="10" t="s">
         <v>225</v>
       </c>
       <c r="D134" s="3" t="s">
@@ -4472,16 +4481,16 @@
       <c r="H134" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I134" s="17"/>
-      <c r="J134" s="19"/>
+      <c r="I134" s="14"/>
+      <c r="J134" s="15"/>
       <c r="K134" s="16"/>
     </row>
     <row r="135" spans="2:11" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="B135" s="15"/>
-      <c r="C135" s="22" t="s">
+      <c r="B135" s="11"/>
+      <c r="C135" s="10" t="s">
         <v>226</v>
       </c>
-      <c r="D135" s="18" t="s">
+      <c r="D135" s="9" t="s">
         <v>216</v>
       </c>
       <c r="E135" s="4" t="s">
@@ -4496,15 +4505,15 @@
       <c r="H135" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I135" s="17"/>
-      <c r="J135" s="19"/>
+      <c r="I135" s="14"/>
+      <c r="J135" s="15"/>
       <c r="K135" s="16"/>
     </row>
     <row r="136" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B136" s="15" t="s">
+      <c r="B136" s="11" t="s">
         <v>237</v>
       </c>
-      <c r="C136" s="21" t="s">
+      <c r="C136" s="12" t="s">
         <v>227</v>
       </c>
       <c r="D136" s="13"/>
@@ -4517,8 +4526,8 @@
       <c r="K136" s="13"/>
     </row>
     <row r="137" spans="2:11" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="B137" s="15"/>
-      <c r="C137" s="22" t="s">
+      <c r="B137" s="11"/>
+      <c r="C137" s="10" t="s">
         <v>238</v>
       </c>
       <c r="D137" s="7" t="s">
@@ -4536,19 +4545,19 @@
       <c r="H137" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="I137" s="17" t="s">
+      <c r="I137" s="25" t="s">
         <v>20</v>
       </c>
-      <c r="J137" s="19" t="s">
+      <c r="J137" s="26" t="s">
         <v>62</v>
       </c>
-      <c r="K137" s="16" t="s">
+      <c r="K137" s="27" t="s">
         <v>235</v>
       </c>
     </row>
     <row r="138" spans="2:11" ht="115.2" x14ac:dyDescent="0.3">
-      <c r="B138" s="15"/>
-      <c r="C138" s="22" t="s">
+      <c r="B138" s="11"/>
+      <c r="C138" s="10" t="s">
         <v>239</v>
       </c>
       <c r="D138" s="3" t="s">
@@ -4566,13 +4575,13 @@
       <c r="H138" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="I138" s="17"/>
-      <c r="J138" s="19"/>
-      <c r="K138" s="16"/>
+      <c r="I138" s="25"/>
+      <c r="J138" s="26"/>
+      <c r="K138" s="27"/>
     </row>
     <row r="139" spans="2:11" ht="72" x14ac:dyDescent="0.3">
-      <c r="B139" s="15"/>
-      <c r="C139" s="22" t="s">
+      <c r="B139" s="11"/>
+      <c r="C139" s="10" t="s">
         <v>240</v>
       </c>
       <c r="D139" s="3" t="s">
@@ -4590,13 +4599,13 @@
       <c r="H139" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I139" s="17"/>
-      <c r="J139" s="19"/>
-      <c r="K139" s="16"/>
+      <c r="I139" s="25"/>
+      <c r="J139" s="26"/>
+      <c r="K139" s="27"/>
     </row>
     <row r="140" spans="2:11" ht="72" x14ac:dyDescent="0.3">
-      <c r="B140" s="15"/>
-      <c r="C140" s="22" t="s">
+      <c r="B140" s="11"/>
+      <c r="C140" s="10" t="s">
         <v>241</v>
       </c>
       <c r="D140" s="3" t="s">
@@ -4614,13 +4623,13 @@
       <c r="H140" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I140" s="17"/>
-      <c r="J140" s="19"/>
-      <c r="K140" s="16"/>
+      <c r="I140" s="25"/>
+      <c r="J140" s="26"/>
+      <c r="K140" s="27"/>
     </row>
     <row r="141" spans="2:11" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="B141" s="15"/>
-      <c r="C141" s="22" t="s">
+      <c r="B141" s="11"/>
+      <c r="C141" s="10" t="s">
         <v>242</v>
       </c>
       <c r="D141" s="3" t="s">
@@ -4638,16 +4647,16 @@
       <c r="H141" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I141" s="17"/>
-      <c r="J141" s="19"/>
-      <c r="K141" s="16"/>
+      <c r="I141" s="25"/>
+      <c r="J141" s="26"/>
+      <c r="K141" s="27"/>
     </row>
     <row r="142" spans="2:11" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B142" s="15"/>
-      <c r="C142" s="22" t="s">
+      <c r="B142" s="11"/>
+      <c r="C142" s="10" t="s">
         <v>243</v>
       </c>
-      <c r="D142" s="18" t="s">
+      <c r="D142" s="9" t="s">
         <v>45</v>
       </c>
       <c r="E142" s="4" t="s">
@@ -4662,13 +4671,13 @@
       <c r="H142" s="8" t="s">
         <v>232</v>
       </c>
-      <c r="I142" s="17"/>
-      <c r="J142" s="19"/>
-      <c r="K142" s="16"/>
+      <c r="I142" s="25"/>
+      <c r="J142" s="26"/>
+      <c r="K142" s="27"/>
     </row>
     <row r="143" spans="2:11" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="B143" s="15"/>
-      <c r="C143" s="22" t="s">
+      <c r="B143" s="11"/>
+      <c r="C143" s="10" t="s">
         <v>244</v>
       </c>
       <c r="D143" s="3" t="s">
@@ -4686,16 +4695,16 @@
       <c r="H143" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I143" s="17"/>
-      <c r="J143" s="19"/>
-      <c r="K143" s="16"/>
+      <c r="I143" s="25"/>
+      <c r="J143" s="26"/>
+      <c r="K143" s="27"/>
     </row>
     <row r="144" spans="2:11" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="B144" s="15"/>
-      <c r="C144" s="22" t="s">
+      <c r="B144" s="11"/>
+      <c r="C144" s="10" t="s">
         <v>245</v>
       </c>
-      <c r="D144" s="18" t="s">
+      <c r="D144" s="9" t="s">
         <v>216</v>
       </c>
       <c r="E144" s="4" t="s">
@@ -4710,47 +4719,12 @@
       <c r="H144" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I144" s="17"/>
-      <c r="J144" s="19"/>
-      <c r="K144" s="16"/>
+      <c r="I144" s="25"/>
+      <c r="J144" s="26"/>
+      <c r="K144" s="27"/>
     </row>
   </sheetData>
   <mergeCells count="49">
-    <mergeCell ref="B136:B144"/>
-    <mergeCell ref="C136:K136"/>
-    <mergeCell ref="I137:I144"/>
-    <mergeCell ref="J137:J144"/>
-    <mergeCell ref="K137:K144"/>
-    <mergeCell ref="B102:B126"/>
-    <mergeCell ref="B127:B135"/>
-    <mergeCell ref="C127:K127"/>
-    <mergeCell ref="I128:I135"/>
-    <mergeCell ref="J128:J135"/>
-    <mergeCell ref="K128:K135"/>
-    <mergeCell ref="C102:K102"/>
-    <mergeCell ref="I103:I126"/>
-    <mergeCell ref="J103:J126"/>
-    <mergeCell ref="K103:K126"/>
-    <mergeCell ref="B84:B101"/>
-    <mergeCell ref="C84:K84"/>
-    <mergeCell ref="I85:I101"/>
-    <mergeCell ref="J85:J101"/>
-    <mergeCell ref="K85:K101"/>
-    <mergeCell ref="B66:B83"/>
-    <mergeCell ref="C66:K66"/>
-    <mergeCell ref="I67:I83"/>
-    <mergeCell ref="J67:J83"/>
-    <mergeCell ref="K67:K83"/>
-    <mergeCell ref="B48:B65"/>
-    <mergeCell ref="C48:K48"/>
-    <mergeCell ref="I49:I65"/>
-    <mergeCell ref="J49:J65"/>
-    <mergeCell ref="K49:K65"/>
-    <mergeCell ref="B30:B47"/>
-    <mergeCell ref="C30:K30"/>
-    <mergeCell ref="I31:I47"/>
-    <mergeCell ref="J31:J47"/>
-    <mergeCell ref="K31:K47"/>
     <mergeCell ref="I12:I29"/>
     <mergeCell ref="J12:J29"/>
     <mergeCell ref="K12:K29"/>
@@ -4765,6 +4739,41 @@
     <mergeCell ref="B10:C10"/>
     <mergeCell ref="C9:K9"/>
     <mergeCell ref="C11:K11"/>
+    <mergeCell ref="B30:B47"/>
+    <mergeCell ref="C30:K30"/>
+    <mergeCell ref="I31:I47"/>
+    <mergeCell ref="J31:J47"/>
+    <mergeCell ref="K31:K47"/>
+    <mergeCell ref="B48:B65"/>
+    <mergeCell ref="C48:K48"/>
+    <mergeCell ref="I49:I65"/>
+    <mergeCell ref="J49:J65"/>
+    <mergeCell ref="K49:K65"/>
+    <mergeCell ref="B66:B83"/>
+    <mergeCell ref="C66:K66"/>
+    <mergeCell ref="I67:I83"/>
+    <mergeCell ref="J67:J83"/>
+    <mergeCell ref="K67:K83"/>
+    <mergeCell ref="B84:B101"/>
+    <mergeCell ref="C84:K84"/>
+    <mergeCell ref="I85:I101"/>
+    <mergeCell ref="J85:J101"/>
+    <mergeCell ref="K85:K101"/>
+    <mergeCell ref="B102:B126"/>
+    <mergeCell ref="B127:B135"/>
+    <mergeCell ref="C127:K127"/>
+    <mergeCell ref="I128:I135"/>
+    <mergeCell ref="J128:J135"/>
+    <mergeCell ref="K128:K135"/>
+    <mergeCell ref="C102:K102"/>
+    <mergeCell ref="I103:I126"/>
+    <mergeCell ref="J103:J126"/>
+    <mergeCell ref="K103:K126"/>
+    <mergeCell ref="B136:B144"/>
+    <mergeCell ref="C136:K136"/>
+    <mergeCell ref="I137:I144"/>
+    <mergeCell ref="J137:J144"/>
+    <mergeCell ref="K137:K144"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>